<commit_message>
fix: Mejorar detección de variantes de productos
- Agregada spec_113 para MiniFuse Recording Pack
- Creada función checkRequiresModelClarification para detectar productos sin modelo específico
- Mejorados mensajes de clarificación para productos con variantes numéricas:
  * MiniFuse: distingue entre 1, 2, 4 y Recording Pack
  * KeyStep: distingue entre KeyStep, 37 y Pro
  * KeyLab: distingue entre Essential, 49, 61 y 88
  * MiniLab: distingue entre versiones
- El bot ahora pregunta específicamente el modelo cuando detecta ambigüedad

Evita confusiones entre líneas de productos y modelos específicos.
</commit_message>
<xml_diff>
--- a/archivos/SoporteBot.xlsx
+++ b/archivos/SoporteBot.xlsx
@@ -1769,7 +1769,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z113"/>
+  <dimension ref="A1:Z114"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="Z31" t="str">
-        <v/>
+        <v>Línea MiniFuse: modelos 1, 2 y 4 disponibles por separado. No incluye micrófono ni auriculares.</v>
       </c>
     </row>
     <row r="32">
@@ -10811,9 +10811,89 @@
         <v/>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>spec_113</v>
+      </c>
+      <c r="B114" t="b">
+        <v>1</v>
+      </c>
+      <c r="C114" t="str">
+        <v>Arturia</v>
+      </c>
+      <c r="D114" t="str">
+        <v>MINIFUSE RECORDING PACK</v>
+      </c>
+      <c r="E114" t="str">
+        <v>minifuse recording pack|arturia minifuse recording pack|minifuse pack|recording pack</v>
+      </c>
+      <c r="F114" t="str">
+        <v>arturia minifuse recording pack</v>
+      </c>
+      <c r="G114" t="str">
+        <v>cosmetic</v>
+      </c>
+      <c r="H114" t="b">
+        <v>1</v>
+      </c>
+      <c r="I114" t="b">
+        <v>1</v>
+      </c>
+      <c r="J114" t="b">
+        <v>1</v>
+      </c>
+      <c r="K114" t="b">
+        <v>1</v>
+      </c>
+      <c r="L114" t="b">
+        <v>1</v>
+      </c>
+      <c r="M114" t="b">
+        <v>1</v>
+      </c>
+      <c r="N114" t="b">
+        <v>0</v>
+      </c>
+      <c r="O114" t="b">
+        <v>0</v>
+      </c>
+      <c r="P114" t="str">
+        <v>line</v>
+      </c>
+      <c r="Q114" t="b">
+        <v>0</v>
+      </c>
+      <c r="R114" t="str">
+        <v>USB-C, MIDI, 2x4 canales, Phantom power 48V, Loopback, 192kHz, incluye micrófono condensador y auriculares</v>
+      </c>
+      <c r="S114" t="str">
+        <v>Sí, el MiniFuse Recording Pack incluye la interfaz MiniFuse 2 que se conecta por USB-C.</v>
+      </c>
+      <c r="T114" t="str">
+        <v>Sí, incluye interfaz MIDI por USB.</v>
+      </c>
+      <c r="U114" t="str">
+        <v>Sí, es una interfaz de audio USB profesional de 2 entradas/4 salidas.</v>
+      </c>
+      <c r="V114" t="str">
+        <v>Sí, requiere instalar drivers de Arturia para la interfaz.</v>
+      </c>
+      <c r="W114" t="str">
+        <v>No, la interfaz no tiene parlantes, pero el pack incluye auriculares profesionales.</v>
+      </c>
+      <c r="X114" t="str">
+        <v>Tiene salidas de línea balanceadas y auriculares. El pack incluye auriculares de monitoreo.</v>
+      </c>
+      <c r="Y114" t="str">
+        <v>https://www.arturia.com/products/audio/minifuse</v>
+      </c>
+      <c r="Z114" t="str">
+        <v>Kit completo: interfaz MiniFuse 2 + micrófono condensador + auriculares</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z113"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z114"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>